<commit_message>
Correções nos gráficos TC_Ext: ajustes de altura, cores e títulos - Corrigido título duplicado no gráfico CPU por Oficina - Ajustada altura dos gráficos para melhor visualização - Corrigida cor da linha pontilhada Flex Bud no gráfico Total por Veículo - Removidos títulos internos dos gráficos para evitar duplicação - Ajustadas alturas: gráficos principais (240px), delta (38px), volume (300px) - Corrigidos rótulos dos gráficos delta para usar mesma cor das barras - Melhorado tratamento de erros e validações nos gráficos
</commit_message>
<xml_diff>
--- a/dados/2025/BUD/df_vol_BUD.xlsx
+++ b/dados/2025/BUD/df_vol_BUD.xlsx
@@ -88,40 +88,40 @@
     <t>CC24 7L</t>
   </si>
   <si>
-    <t>janeiro</t>
+    <t>Janeiro</t>
   </si>
   <si>
-    <t>fevereiro</t>
+    <t>Fevereiro</t>
   </si>
   <si>
-    <t>março</t>
+    <t>Março</t>
   </si>
   <si>
-    <t>abril</t>
+    <t>Abril</t>
   </si>
   <si>
-    <t>maio</t>
+    <t>Maio</t>
   </si>
   <si>
-    <t>junho</t>
+    <t>Junho</t>
   </si>
   <si>
-    <t>julho</t>
+    <t>Julho</t>
   </si>
   <si>
-    <t>agosto</t>
+    <t>Agosto</t>
   </si>
   <si>
-    <t>setembro</t>
+    <t>Setembro</t>
   </si>
   <si>
-    <t>outubro</t>
+    <t>Outubro</t>
   </si>
   <si>
-    <t>novembro</t>
+    <t>Novembro</t>
   </si>
   <si>
-    <t>dezembro</t>
+    <t>Dezembro</t>
   </si>
 </sst>
 </file>

</xml_diff>